<commit_message>
Fixed Problems with seed from csv
</commit_message>
<xml_diff>
--- a/ITech/ProductsDetails.xlsx
+++ b/ITech/ProductsDetails.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workspace\GraduationProject\ITech\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D59D411E-E532-4BE9-A539-9C0DE44432BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22AE70CE-95E3-467D-9437-BC8D8A6AFE4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="16200" windowHeight="9360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>ITSIN</t>
   </si>
@@ -64,6 +64,27 @@
   </si>
   <si>
     <t>Graphics Processor: NVIDIA® GeForce® MX330</t>
+  </si>
+  <si>
+    <t>IT-CSV-2</t>
+  </si>
+  <si>
+    <t>title2.1</t>
+  </si>
+  <si>
+    <t>title2.2</t>
+  </si>
+  <si>
+    <t>title2.3</t>
+  </si>
+  <si>
+    <t>content2.1</t>
+  </si>
+  <si>
+    <t>content2.2</t>
+  </si>
+  <si>
+    <t>content2.3</t>
   </si>
 </sst>
 </file>
@@ -391,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -442,7 +463,37 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
+      <c r="A5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added data to productDetails
</commit_message>
<xml_diff>
--- a/ITech/ProductsDetails.xlsx
+++ b/ITech/ProductsDetails.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\workspace\GraduationProject\ITech\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{370FB01E-0784-4A57-857A-A966DD9E9101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5A40FD-3491-41AD-A09D-BF4AC60AB5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>ITSIN</t>
   </si>
@@ -43,6 +43,51 @@
   </si>
   <si>
     <t>Content</t>
+  </si>
+  <si>
+    <t>Network</t>
+  </si>
+  <si>
+    <t>IT-CSV-1</t>
+  </si>
+  <si>
+    <t>GSM / HSPA / LTE</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <r>
+      <t>Type</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: LCD, 90Hz</t>
+    </r>
+  </si>
+  <si>
+    <t>Platform</t>
+  </si>
+  <si>
+    <r>
+      <t>OS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Android 11, MIUI 12.5</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -387,6 +432,39 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
     </row>

</xml_diff>